<commit_message>
docs: document multi-environment execution
</commit_message>
<xml_diff>
--- a/data/test_cases_template.xlsx
+++ b/data/test_cases_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R413ce86d7cf34249"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="Rae3ff5326dcd462b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R072fc47b4efb4d10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R5d4c602352ed452a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -564,7 +564,7 @@
         <x:v>smoke,p0</x:v>
       </x:c>
       <x:c r="M2" s="19" t="str">
-        <x:v>Clean app database; onboarding completed with Kimbal, US Dollar, monthly budget 30000, and Bank SMS Reader enabled; user is on the Home page</x:v>
+        <x:v>Clean app database; onboarding completed with the selected environment profile, US Dollar, monthly budget 30000, and configured Bank SMS Reader state; user is on the Home page</x:v>
       </x:c>
       <x:c r="N2" s="19" t="str">
         <x:v>user taps "Add Expense"
@@ -619,7 +619,7 @@
         <x:v>smoke,p0</x:v>
       </x:c>
       <x:c r="M3" s="18" t="str">
-        <x:v>Clean app database; onboarding completed with Kimbal, US Dollar, monthly budget 30000, and Bank SMS Reader enabled; user is on the Home page</x:v>
+        <x:v>Clean app database; onboarding completed with the selected environment profile, US Dollar, monthly budget 30000, and configured Bank SMS Reader state; user is on the Home page</x:v>
       </x:c>
       <x:c r="N3" s="18" t="str">
         <x:v>user taps "Add Income"
@@ -673,7 +673,7 @@
         <x:v>smoke,p0</x:v>
       </x:c>
       <x:c r="M4" s="20" t="str">
-        <x:v>Clean app database; onboarding completed with Kimbal, US Dollar, monthly budget 30000, and Bank SMS Reader enabled; user is on the Home page</x:v>
+        <x:v>Clean app database; onboarding completed with the selected environment profile, US Dollar, monthly budget 30000, and configured Bank SMS Reader state; user is on the Home page</x:v>
       </x:c>
       <x:c r="N4" s="20" t="str">
         <x:v>user taps "Add Transfer"
@@ -727,7 +727,7 @@
         <x:v>smoke,p0</x:v>
       </x:c>
       <x:c r="M5" s="18" t="str">
-        <x:v>Clean app database; onboarding completed with Kimbal, US Dollar, monthly budget 30000, and Bank SMS Reader enabled; user is on the Home page</x:v>
+        <x:v>Clean app database; onboarding completed with the selected environment profile, US Dollar, monthly budget 30000, and configured Bank SMS Reader state; user is on the Home page</x:v>
       </x:c>
       <x:c r="N5" s="18" t="str">
         <x:v>user taps "Add Expense"
@@ -781,7 +781,7 @@
         <x:v>p1,custom_category</x:v>
       </x:c>
       <x:c r="M6" s="20" t="str">
-        <x:v>Clean app database; onboarding completed with Kimbal, US Dollar, monthly budget 30000, and Bank SMS Reader enabled; user is on the Home page</x:v>
+        <x:v>Clean app database; onboarding completed with the selected environment profile, US Dollar, monthly budget 30000, and configured Bank SMS Reader state; user is on the Home page</x:v>
       </x:c>
       <x:c r="N6" s="20" t="str">
         <x:v>user taps "Add Expense"
@@ -837,7 +837,7 @@
         <x:v>p1,filter</x:v>
       </x:c>
       <x:c r="M7" s="18" t="str">
-        <x:v>Clean app database; onboarding completed with Kimbal, US Dollar, monthly budget 30000, and Bank SMS Reader enabled; user is on the Home page</x:v>
+        <x:v>Clean app database; onboarding completed with the selected environment profile, US Dollar, monthly budget 30000, and configured Bank SMS Reader state; user is on the Home page</x:v>
       </x:c>
       <x:c r="N7" s="18" t="str">
         <x:v>user taps "Add Expense"
@@ -896,7 +896,7 @@
         <x:v>p1,grouping</x:v>
       </x:c>
       <x:c r="M8" s="20" t="str">
-        <x:v>Clean app database; onboarding completed with Kimbal, US Dollar, monthly budget 30000, and Bank SMS Reader enabled; user is on the Home page</x:v>
+        <x:v>Clean app database; onboarding completed with the selected environment profile, US Dollar, monthly budget 30000, and configured Bank SMS Reader state; user is on the Home page</x:v>
       </x:c>
       <x:c r="N8" s="20" t="str">
         <x:v>user taps "Add Expense"
@@ -931,7 +931,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3ca2f518a5e4924"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6a2a32c45794cc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>